<commit_message>
Ajouter fiche évaluation coach PSG Academy + optimiser impression
- Nouvelle fiche coach PSG Academy (HTML + Excel) avec DA PSG
  (bleu #0C1C3E, rouge #E30613, bg-psg.jpg)
- 5 catégories coach : Préparation, Pédagogie, Communication,
  Gestion du groupe, Sécurité & Attitude
- Optimiser impression 1 page A4 portrait (arbitre HTML + Excel)
- Ajouter evaluation-coach.html au workflow GitHub Pages

https://claude.ai/code/session_01ELsd82FqhFHd9QHcP9yAqq
</commit_message>
<xml_diff>
--- a/Evaluation Arbitre - UrbanSoccer.xlsx
+++ b/Evaluation Arbitre - UrbanSoccer.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Évaluation Arbitre" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Évaluation Arbitre'!$A$1:$H$70</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Évaluation Arbitre'!$A$1:$H$65</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,13 +31,13 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="16"/>
+      <sz val="14"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FF6600"/>
-      <sz val="9"/>
+      <sz val="8"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -59,8 +59,14 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="00888888"/>
+      <sz val="7"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="00FF6600"/>
-      <sz val="8"/>
+      <sz val="7"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -69,20 +75,31 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <color rgb="00888888"/>
+      <sz val="6"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="004CAF50"/>
       <sz val="7"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="004CAF50"/>
-      <sz val="8"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
       <color rgb="00FF9800"/>
-      <sz val="8"/>
+      <sz val="7"/>
     </font>
   </fonts>
   <fills count="7">
@@ -248,7 +265,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -269,50 +286,53 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -679,7 +699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H70"/>
+  <dimension ref="A1:H69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -692,21 +712,21 @@
     <col width="5" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
+    <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>ÉVALUATION ARBITRE</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="16" customHeight="1">
+    <row r="2" ht="13" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>UrbanSoccer</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="3" customHeight="1">
+    <row r="3" ht="2" customHeight="1">
       <c r="A3" s="3" t="n"/>
       <c r="B3" s="3" t="n"/>
       <c r="C3" s="3" t="n"/>
@@ -716,7 +736,7 @@
       <c r="G3" s="3" t="n"/>
       <c r="H3" s="3" t="n"/>
     </row>
-    <row r="4" ht="18" customHeight="1">
+    <row r="4" ht="14" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>INFORMATIONS</t>
@@ -730,7 +750,7 @@
       <c r="G4" s="5" t="n"/>
       <c r="H4" s="5" t="n"/>
     </row>
-    <row r="5" ht="22" customHeight="1">
+    <row r="5" ht="18" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Arbitre</t>
@@ -748,7 +768,7 @@
       <c r="G5" s="8" t="n"/>
       <c r="H5" s="9" t="n"/>
     </row>
-    <row r="6" ht="22" customHeight="1">
+    <row r="6" ht="18" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Match</t>
@@ -762,7 +782,7 @@
       <c r="G6" s="8" t="n"/>
       <c r="H6" s="9" t="n"/>
     </row>
-    <row r="7" ht="22" customHeight="1">
+    <row r="7" ht="18" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Créneau</t>
@@ -780,700 +800,713 @@
       <c r="G7" s="8" t="n"/>
       <c r="H7" s="9" t="n"/>
     </row>
-    <row r="8">
-      <c r="A8" s="10" t="n"/>
-      <c r="B8" s="10" t="n"/>
-      <c r="C8" s="10" t="n"/>
-      <c r="D8" s="10" t="n"/>
-      <c r="E8" s="10" t="n"/>
-      <c r="F8" s="10" t="n"/>
-      <c r="G8" s="10" t="n"/>
-      <c r="H8" s="10" t="n"/>
-    </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+    <row r="8" ht="14" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>ÉVALUATION</t>
         </is>
       </c>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
-    </row>
-    <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="B8" s="5" t="n"/>
+      <c r="C8" s="5" t="n"/>
+      <c r="D8" s="5" t="n"/>
+      <c r="E8" s="5" t="n"/>
+      <c r="F8" s="5" t="n"/>
+      <c r="G8" s="5" t="n"/>
+      <c r="H8" s="5" t="n"/>
+    </row>
+    <row r="9" ht="13" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Critère</t>
         </is>
       </c>
-      <c r="C10" s="12" t="inlineStr">
+      <c r="C9" s="11" t="inlineStr">
         <is>
           <t>N/N</t>
         </is>
       </c>
-      <c r="D10" s="12" t="inlineStr">
+      <c r="D9" s="11" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E10" s="12" t="inlineStr">
+      <c r="E9" s="11" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="F10" s="12" t="inlineStr">
+      <c r="F9" s="11" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="G10" s="12" t="inlineStr">
+      <c r="G9" s="11" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="H10" s="12" t="inlineStr">
+      <c r="H9" s="11" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="13" t="inlineStr">
+    <row r="10" ht="13" customHeight="1">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>PLACEMENT &amp; DÉPLACEMENTS</t>
         </is>
       </c>
-      <c r="B11" s="14" t="n"/>
-      <c r="C11" s="14" t="n"/>
-      <c r="D11" s="14" t="n"/>
-      <c r="E11" s="14" t="n"/>
-      <c r="F11" s="14" t="n"/>
-      <c r="G11" s="14" t="n"/>
-      <c r="H11" s="14" t="n"/>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="15" t="inlineStr">
+      <c r="B10" s="13" t="n"/>
+      <c r="C10" s="13" t="n"/>
+      <c r="D10" s="13" t="n"/>
+      <c r="E10" s="13" t="n"/>
+      <c r="F10" s="13" t="n"/>
+      <c r="G10" s="13" t="n"/>
+      <c r="H10" s="13" t="n"/>
+    </row>
+    <row r="11" ht="15" customHeight="1">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>Placement &amp; Déplacements</t>
         </is>
       </c>
-      <c r="C12" s="16" t="inlineStr"/>
-      <c r="D12" s="16" t="inlineStr"/>
-      <c r="E12" s="16" t="inlineStr"/>
-      <c r="F12" s="16" t="inlineStr"/>
-      <c r="G12" s="16" t="inlineStr"/>
-      <c r="H12" s="16" t="inlineStr"/>
+      <c r="C11" s="15" t="inlineStr"/>
+      <c r="D11" s="15" t="inlineStr"/>
+      <c r="E11" s="15" t="inlineStr"/>
+      <c r="F11" s="15" t="inlineStr"/>
+      <c r="G11" s="15" t="inlineStr"/>
+      <c r="H11" s="15" t="inlineStr"/>
+    </row>
+    <row r="12" ht="10" customHeight="1">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>Positionnement, déplacements fluides, bons angles de vision</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="13" customHeight="1">
-      <c r="A13" s="17" t="inlineStr">
-        <is>
-          <t>Positionnement, déplacements fluides, bons angles de vision</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>SIFFLET &amp; SIGNALÉTIQUE</t>
         </is>
       </c>
-      <c r="B14" s="14" t="n"/>
-      <c r="C14" s="14" t="n"/>
-      <c r="D14" s="14" t="n"/>
-      <c r="E14" s="14" t="n"/>
-      <c r="F14" s="14" t="n"/>
-      <c r="G14" s="14" t="n"/>
-      <c r="H14" s="14" t="n"/>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="18" t="inlineStr">
+      <c r="B13" s="13" t="n"/>
+      <c r="C13" s="13" t="n"/>
+      <c r="D13" s="13" t="n"/>
+      <c r="E13" s="13" t="n"/>
+      <c r="F13" s="13" t="n"/>
+      <c r="G13" s="13" t="n"/>
+      <c r="H13" s="13" t="n"/>
+    </row>
+    <row r="14" ht="15" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t>Clarté du sifflet</t>
         </is>
       </c>
-      <c r="C15" s="19" t="inlineStr"/>
-      <c r="D15" s="19" t="inlineStr"/>
-      <c r="E15" s="19" t="inlineStr"/>
-      <c r="F15" s="19" t="inlineStr"/>
-      <c r="G15" s="19" t="inlineStr"/>
-      <c r="H15" s="19" t="inlineStr"/>
-    </row>
-    <row r="16" ht="13" customHeight="1">
-      <c r="A16" s="20" t="inlineStr">
+      <c r="C14" s="18" t="inlineStr"/>
+      <c r="D14" s="18" t="inlineStr"/>
+      <c r="E14" s="18" t="inlineStr"/>
+      <c r="F14" s="18" t="inlineStr"/>
+      <c r="G14" s="18" t="inlineStr"/>
+      <c r="H14" s="18" t="inlineStr"/>
+    </row>
+    <row r="15" ht="10" customHeight="1">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>Coups de sifflet nets, audibles et bien différenciés</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="15" t="inlineStr">
+    <row r="16" ht="15" customHeight="1">
+      <c r="A16" s="14" t="inlineStr">
         <is>
           <t>Gestuelle</t>
         </is>
       </c>
-      <c r="C17" s="16" t="inlineStr"/>
-      <c r="D17" s="16" t="inlineStr"/>
-      <c r="E17" s="16" t="inlineStr"/>
-      <c r="F17" s="16" t="inlineStr"/>
-      <c r="G17" s="16" t="inlineStr"/>
-      <c r="H17" s="16" t="inlineStr"/>
-    </row>
-    <row r="18" ht="13" customHeight="1">
+      <c r="C16" s="15" t="inlineStr"/>
+      <c r="D16" s="15" t="inlineStr"/>
+      <c r="E16" s="15" t="inlineStr"/>
+      <c r="F16" s="15" t="inlineStr"/>
+      <c r="G16" s="15" t="inlineStr"/>
+      <c r="H16" s="15" t="inlineStr"/>
+    </row>
+    <row r="17" ht="10" customHeight="1">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>Signale clairement les décisions (fautes, touches, corners, coups francs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1">
       <c r="A18" s="17" t="inlineStr">
         <is>
-          <t>Signale clairement les décisions (fautes, touches, corners, coups francs)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="18" t="inlineStr">
-        <is>
           <t>Timing du sifflet</t>
         </is>
       </c>
-      <c r="C19" s="19" t="inlineStr"/>
-      <c r="D19" s="19" t="inlineStr"/>
-      <c r="E19" s="19" t="inlineStr"/>
-      <c r="F19" s="19" t="inlineStr"/>
-      <c r="G19" s="19" t="inlineStr"/>
-      <c r="H19" s="19" t="inlineStr"/>
+      <c r="C18" s="18" t="inlineStr"/>
+      <c r="D18" s="18" t="inlineStr"/>
+      <c r="E18" s="18" t="inlineStr"/>
+      <c r="F18" s="18" t="inlineStr"/>
+      <c r="G18" s="18" t="inlineStr"/>
+      <c r="H18" s="18" t="inlineStr"/>
+    </row>
+    <row r="19" ht="10" customHeight="1">
+      <c r="A19" s="19" t="inlineStr">
+        <is>
+          <t>Siffle au bon moment, ni trop tôt ni trop tard</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="13" customHeight="1">
-      <c r="A20" s="20" t="inlineStr">
-        <is>
-          <t>Siffle au bon moment, ni trop tôt ni trop tard</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="13" t="inlineStr">
+      <c r="A20" s="12" t="inlineStr">
         <is>
           <t>DÉCISIONS &amp; LECTURE DU JEU</t>
         </is>
       </c>
-      <c r="B21" s="14" t="n"/>
-      <c r="C21" s="14" t="n"/>
-      <c r="D21" s="14" t="n"/>
-      <c r="E21" s="14" t="n"/>
-      <c r="F21" s="14" t="n"/>
-      <c r="G21" s="14" t="n"/>
-      <c r="H21" s="14" t="n"/>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="15" t="inlineStr">
+      <c r="B20" s="13" t="n"/>
+      <c r="C20" s="13" t="n"/>
+      <c r="D20" s="13" t="n"/>
+      <c r="E20" s="13" t="n"/>
+      <c r="F20" s="13" t="n"/>
+      <c r="G20" s="13" t="n"/>
+      <c r="H20" s="13" t="n"/>
+    </row>
+    <row r="21" ht="15" customHeight="1">
+      <c r="A21" s="14" t="inlineStr">
         <is>
           <t>Justesse des décisions</t>
         </is>
       </c>
-      <c r="C22" s="16" t="inlineStr"/>
-      <c r="D22" s="16" t="inlineStr"/>
-      <c r="E22" s="16" t="inlineStr"/>
-      <c r="F22" s="16" t="inlineStr"/>
-      <c r="G22" s="16" t="inlineStr"/>
-      <c r="H22" s="16" t="inlineStr"/>
-    </row>
-    <row r="23" ht="13" customHeight="1">
+      <c r="C21" s="15" t="inlineStr"/>
+      <c r="D21" s="15" t="inlineStr"/>
+      <c r="E21" s="15" t="inlineStr"/>
+      <c r="F21" s="15" t="inlineStr"/>
+      <c r="G21" s="15" t="inlineStr"/>
+      <c r="H21" s="15" t="inlineStr"/>
+    </row>
+    <row r="22" ht="10" customHeight="1">
+      <c r="A22" s="16" t="inlineStr">
+        <is>
+          <t>Les décisions prises sont correctes et cohérentes</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15" customHeight="1">
       <c r="A23" s="17" t="inlineStr">
         <is>
-          <t>Les décisions prises sont correctes et cohérentes</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="18" t="inlineStr">
-        <is>
           <t>Cohérence</t>
         </is>
       </c>
-      <c r="C24" s="19" t="inlineStr"/>
-      <c r="D24" s="19" t="inlineStr"/>
-      <c r="E24" s="19" t="inlineStr"/>
-      <c r="F24" s="19" t="inlineStr"/>
-      <c r="G24" s="19" t="inlineStr"/>
-      <c r="H24" s="19" t="inlineStr"/>
-    </row>
-    <row r="25" ht="13" customHeight="1">
-      <c r="A25" s="20" t="inlineStr">
+      <c r="C23" s="18" t="inlineStr"/>
+      <c r="D23" s="18" t="inlineStr"/>
+      <c r="E23" s="18" t="inlineStr"/>
+      <c r="F23" s="18" t="inlineStr"/>
+      <c r="G23" s="18" t="inlineStr"/>
+      <c r="H23" s="18" t="inlineStr"/>
+    </row>
+    <row r="24" ht="10" customHeight="1">
+      <c r="A24" s="19" t="inlineStr">
         <is>
           <t>Mêmes critères du début à la fin du match</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="15" t="inlineStr">
+    <row r="25" ht="15" customHeight="1">
+      <c r="A25" s="14" t="inlineStr">
         <is>
           <t>Gestion de l'avantage</t>
         </is>
       </c>
-      <c r="C26" s="16" t="inlineStr"/>
-      <c r="D26" s="16" t="inlineStr"/>
-      <c r="E26" s="16" t="inlineStr"/>
-      <c r="F26" s="16" t="inlineStr"/>
-      <c r="G26" s="16" t="inlineStr"/>
-      <c r="H26" s="16" t="inlineStr"/>
-    </row>
-    <row r="27" ht="13" customHeight="1">
+      <c r="C25" s="15" t="inlineStr"/>
+      <c r="D25" s="15" t="inlineStr"/>
+      <c r="E25" s="15" t="inlineStr"/>
+      <c r="F25" s="15" t="inlineStr"/>
+      <c r="G25" s="15" t="inlineStr"/>
+      <c r="H25" s="15" t="inlineStr"/>
+    </row>
+    <row r="26" ht="10" customHeight="1">
+      <c r="A26" s="16" t="inlineStr">
+        <is>
+          <t>Laisse jouer quand c'est pertinent, laisse le jeu couler</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="15" customHeight="1">
       <c r="A27" s="17" t="inlineStr">
         <is>
-          <t>Laisse jouer quand c'est pertinent, laisse le jeu couler</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="18" t="inlineStr">
-        <is>
           <t>Connaissance des règles</t>
         </is>
       </c>
-      <c r="C28" s="19" t="inlineStr"/>
-      <c r="D28" s="19" t="inlineStr"/>
-      <c r="E28" s="19" t="inlineStr"/>
-      <c r="F28" s="19" t="inlineStr"/>
-      <c r="G28" s="19" t="inlineStr"/>
-      <c r="H28" s="19" t="inlineStr"/>
+      <c r="C27" s="18" t="inlineStr"/>
+      <c r="D27" s="18" t="inlineStr"/>
+      <c r="E27" s="18" t="inlineStr"/>
+      <c r="F27" s="18" t="inlineStr"/>
+      <c r="G27" s="18" t="inlineStr"/>
+      <c r="H27" s="18" t="inlineStr"/>
+    </row>
+    <row r="28" ht="10" customHeight="1">
+      <c r="A28" s="19" t="inlineStr">
+        <is>
+          <t>Maîtrise les règles spécifiques UrbanSoccer / futsal</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="13" customHeight="1">
-      <c r="A29" s="20" t="inlineStr">
-        <is>
-          <t>Maîtrise les règles spécifiques UrbanSoccer / futsal</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="16" customHeight="1">
-      <c r="A30" s="13" t="inlineStr">
+      <c r="A29" s="12" t="inlineStr">
         <is>
           <t>COMMUNICATION &amp; GESTION</t>
         </is>
       </c>
-      <c r="B30" s="14" t="n"/>
-      <c r="C30" s="14" t="n"/>
-      <c r="D30" s="14" t="n"/>
-      <c r="E30" s="14" t="n"/>
-      <c r="F30" s="14" t="n"/>
-      <c r="G30" s="14" t="n"/>
-      <c r="H30" s="14" t="n"/>
-    </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="15" t="inlineStr">
+      <c r="B29" s="13" t="n"/>
+      <c r="C29" s="13" t="n"/>
+      <c r="D29" s="13" t="n"/>
+      <c r="E29" s="13" t="n"/>
+      <c r="F29" s="13" t="n"/>
+      <c r="G29" s="13" t="n"/>
+      <c r="H29" s="13" t="n"/>
+    </row>
+    <row r="30" ht="15" customHeight="1">
+      <c r="A30" s="14" t="inlineStr">
         <is>
           <t>Communication joueurs</t>
         </is>
       </c>
-      <c r="C31" s="16" t="inlineStr"/>
-      <c r="D31" s="16" t="inlineStr"/>
-      <c r="E31" s="16" t="inlineStr"/>
-      <c r="F31" s="16" t="inlineStr"/>
-      <c r="G31" s="16" t="inlineStr"/>
-      <c r="H31" s="16" t="inlineStr"/>
-    </row>
-    <row r="32" ht="13" customHeight="1">
+      <c r="C30" s="15" t="inlineStr"/>
+      <c r="D30" s="15" t="inlineStr"/>
+      <c r="E30" s="15" t="inlineStr"/>
+      <c r="F30" s="15" t="inlineStr"/>
+      <c r="G30" s="15" t="inlineStr"/>
+      <c r="H30" s="15" t="inlineStr"/>
+    </row>
+    <row r="31" ht="10" customHeight="1">
+      <c r="A31" s="16" t="inlineStr">
+        <is>
+          <t>Échange calmement, explique ses décisions</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="15" customHeight="1">
       <c r="A32" s="17" t="inlineStr">
         <is>
-          <t>Échange calmement, explique ses décisions</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="18" t="inlineStr">
-        <is>
           <t>Autorité &amp; Présence</t>
         </is>
       </c>
-      <c r="C33" s="19" t="inlineStr"/>
-      <c r="D33" s="19" t="inlineStr"/>
-      <c r="E33" s="19" t="inlineStr"/>
-      <c r="F33" s="19" t="inlineStr"/>
-      <c r="G33" s="19" t="inlineStr"/>
-      <c r="H33" s="19" t="inlineStr"/>
-    </row>
-    <row r="34" ht="13" customHeight="1">
-      <c r="A34" s="20" t="inlineStr">
+      <c r="C32" s="18" t="inlineStr"/>
+      <c r="D32" s="18" t="inlineStr"/>
+      <c r="E32" s="18" t="inlineStr"/>
+      <c r="F32" s="18" t="inlineStr"/>
+      <c r="G32" s="18" t="inlineStr"/>
+      <c r="H32" s="18" t="inlineStr"/>
+    </row>
+    <row r="33" ht="10" customHeight="1">
+      <c r="A33" s="19" t="inlineStr">
         <is>
           <t>Inspire le respect, contrôle le match sans être autoritaire</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="15" t="inlineStr">
+    <row r="34" ht="15" customHeight="1">
+      <c r="A34" s="14" t="inlineStr">
         <is>
           <t>Gestion des tensions</t>
         </is>
       </c>
-      <c r="C35" s="16" t="inlineStr"/>
-      <c r="D35" s="16" t="inlineStr"/>
-      <c r="E35" s="16" t="inlineStr"/>
-      <c r="F35" s="16" t="inlineStr"/>
-      <c r="G35" s="16" t="inlineStr"/>
-      <c r="H35" s="16" t="inlineStr"/>
-    </row>
-    <row r="36" ht="13" customHeight="1">
+      <c r="C34" s="15" t="inlineStr"/>
+      <c r="D34" s="15" t="inlineStr"/>
+      <c r="E34" s="15" t="inlineStr"/>
+      <c r="F34" s="15" t="inlineStr"/>
+      <c r="G34" s="15" t="inlineStr"/>
+      <c r="H34" s="15" t="inlineStr"/>
+    </row>
+    <row r="35" ht="10" customHeight="1">
+      <c r="A35" s="16" t="inlineStr">
+        <is>
+          <t>Désamorce les situations conflictuelles avec sang-froid</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="15" customHeight="1">
       <c r="A36" s="17" t="inlineStr">
         <is>
-          <t>Désamorce les situations conflictuelles avec sang-froid</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="18" t="inlineStr">
-        <is>
           <t>Utilisation des sanctions</t>
         </is>
       </c>
-      <c r="C37" s="19" t="inlineStr"/>
-      <c r="D37" s="19" t="inlineStr"/>
-      <c r="E37" s="19" t="inlineStr"/>
-      <c r="F37" s="19" t="inlineStr"/>
-      <c r="G37" s="19" t="inlineStr"/>
-      <c r="H37" s="19" t="inlineStr"/>
+      <c r="C36" s="18" t="inlineStr"/>
+      <c r="D36" s="18" t="inlineStr"/>
+      <c r="E36" s="18" t="inlineStr"/>
+      <c r="F36" s="18" t="inlineStr"/>
+      <c r="G36" s="18" t="inlineStr"/>
+      <c r="H36" s="18" t="inlineStr"/>
+    </row>
+    <row r="37" ht="10" customHeight="1">
+      <c r="A37" s="19" t="inlineStr">
+        <is>
+          <t>Avertissements et cartons justes et proportionnés</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="13" customHeight="1">
-      <c r="A38" s="20" t="inlineStr">
-        <is>
-          <t>Avertissements et cartons justes et proportionnés</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="16" customHeight="1">
-      <c r="A39" s="13" t="inlineStr">
+      <c r="A38" s="12" t="inlineStr">
         <is>
           <t>ATTITUDE &amp; PROFESSIONNALISME</t>
         </is>
       </c>
-      <c r="B39" s="14" t="n"/>
-      <c r="C39" s="14" t="n"/>
-      <c r="D39" s="14" t="n"/>
-      <c r="E39" s="14" t="n"/>
-      <c r="F39" s="14" t="n"/>
-      <c r="G39" s="14" t="n"/>
-      <c r="H39" s="14" t="n"/>
-    </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="15" t="inlineStr">
+      <c r="B38" s="13" t="n"/>
+      <c r="C38" s="13" t="n"/>
+      <c r="D38" s="13" t="n"/>
+      <c r="E38" s="13" t="n"/>
+      <c r="F38" s="13" t="n"/>
+      <c r="G38" s="13" t="n"/>
+      <c r="H38" s="13" t="n"/>
+    </row>
+    <row r="39" ht="15" customHeight="1">
+      <c r="A39" s="14" t="inlineStr">
         <is>
           <t>Présentation</t>
         </is>
       </c>
-      <c r="C40" s="16" t="inlineStr"/>
-      <c r="D40" s="16" t="inlineStr"/>
-      <c r="E40" s="16" t="inlineStr"/>
-      <c r="F40" s="16" t="inlineStr"/>
-      <c r="G40" s="16" t="inlineStr"/>
-      <c r="H40" s="16" t="inlineStr"/>
-    </row>
-    <row r="41" ht="13" customHeight="1">
+      <c r="C39" s="15" t="inlineStr"/>
+      <c r="D39" s="15" t="inlineStr"/>
+      <c r="E39" s="15" t="inlineStr"/>
+      <c r="F39" s="15" t="inlineStr"/>
+      <c r="G39" s="15" t="inlineStr"/>
+      <c r="H39" s="15" t="inlineStr"/>
+    </row>
+    <row r="40" ht="10" customHeight="1">
+      <c r="A40" s="16" t="inlineStr">
+        <is>
+          <t>Tenue correcte, ponctualité, équipement d'arbitre</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="15" customHeight="1">
       <c r="A41" s="17" t="inlineStr">
         <is>
-          <t>Tenue correcte, ponctualité, équipement d'arbitre</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="18" t="inlineStr">
-        <is>
           <t>Impartialité</t>
         </is>
       </c>
-      <c r="C42" s="19" t="inlineStr"/>
-      <c r="D42" s="19" t="inlineStr"/>
-      <c r="E42" s="19" t="inlineStr"/>
-      <c r="F42" s="19" t="inlineStr"/>
-      <c r="G42" s="19" t="inlineStr"/>
-      <c r="H42" s="19" t="inlineStr"/>
-    </row>
-    <row r="43" ht="13" customHeight="1">
-      <c r="A43" s="20" t="inlineStr">
+      <c r="C41" s="18" t="inlineStr"/>
+      <c r="D41" s="18" t="inlineStr"/>
+      <c r="E41" s="18" t="inlineStr"/>
+      <c r="F41" s="18" t="inlineStr"/>
+      <c r="G41" s="18" t="inlineStr"/>
+      <c r="H41" s="18" t="inlineStr"/>
+    </row>
+    <row r="42" ht="10" customHeight="1">
+      <c r="A42" s="19" t="inlineStr">
         <is>
           <t>Traite les deux équipes de façon équitable</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="20" customHeight="1">
-      <c r="A44" s="15" t="inlineStr">
+    <row r="43" ht="15" customHeight="1">
+      <c r="A43" s="14" t="inlineStr">
         <is>
           <t>Concentration</t>
         </is>
       </c>
-      <c r="C44" s="16" t="inlineStr"/>
-      <c r="D44" s="16" t="inlineStr"/>
-      <c r="E44" s="16" t="inlineStr"/>
-      <c r="F44" s="16" t="inlineStr"/>
-      <c r="G44" s="16" t="inlineStr"/>
-      <c r="H44" s="16" t="inlineStr"/>
-    </row>
-    <row r="45" ht="13" customHeight="1">
+      <c r="C43" s="15" t="inlineStr"/>
+      <c r="D43" s="15" t="inlineStr"/>
+      <c r="E43" s="15" t="inlineStr"/>
+      <c r="F43" s="15" t="inlineStr"/>
+      <c r="G43" s="15" t="inlineStr"/>
+      <c r="H43" s="15" t="inlineStr"/>
+    </row>
+    <row r="44" ht="10" customHeight="1">
+      <c r="A44" s="16" t="inlineStr">
+        <is>
+          <t>Reste attentif du début à la fin, même sur les temps morts</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="15" customHeight="1">
       <c r="A45" s="17" t="inlineStr">
         <is>
-          <t>Reste attentif du début à la fin, même sur les temps morts</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="20" customHeight="1">
-      <c r="A46" s="18" t="inlineStr">
-        <is>
           <t>Timing &amp; Gestion du temps</t>
         </is>
       </c>
-      <c r="C46" s="19" t="inlineStr"/>
-      <c r="D46" s="19" t="inlineStr"/>
-      <c r="E46" s="19" t="inlineStr"/>
-      <c r="F46" s="19" t="inlineStr"/>
-      <c r="G46" s="19" t="inlineStr"/>
-      <c r="H46" s="19" t="inlineStr"/>
+      <c r="C45" s="18" t="inlineStr"/>
+      <c r="D45" s="18" t="inlineStr"/>
+      <c r="E45" s="18" t="inlineStr"/>
+      <c r="F45" s="18" t="inlineStr"/>
+      <c r="G45" s="18" t="inlineStr"/>
+      <c r="H45" s="18" t="inlineStr"/>
+    </row>
+    <row r="46" ht="10" customHeight="1">
+      <c r="A46" s="19" t="inlineStr">
+        <is>
+          <t>Début des matchs à l'heure, durées de mi-temps, enchaînement</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="13" customHeight="1">
-      <c r="A47" s="20" t="inlineStr">
-        <is>
-          <t>Début des matchs à l'heure, durées de mi-temps, enchaînement</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="16" customHeight="1">
-      <c r="A48" s="13" t="inlineStr">
+      <c r="A47" s="12" t="inlineStr">
         <is>
           <t>ANIMATION</t>
         </is>
       </c>
-      <c r="B48" s="14" t="n"/>
-      <c r="C48" s="14" t="n"/>
-      <c r="D48" s="14" t="n"/>
-      <c r="E48" s="14" t="n"/>
-      <c r="F48" s="14" t="n"/>
-      <c r="G48" s="14" t="n"/>
-      <c r="H48" s="14" t="n"/>
-    </row>
-    <row r="49" ht="20" customHeight="1">
-      <c r="A49" s="15" t="inlineStr">
+      <c r="B47" s="13" t="n"/>
+      <c r="C47" s="13" t="n"/>
+      <c r="D47" s="13" t="n"/>
+      <c r="E47" s="13" t="n"/>
+      <c r="F47" s="13" t="n"/>
+      <c r="G47" s="13" t="n"/>
+      <c r="H47" s="13" t="n"/>
+    </row>
+    <row r="48" ht="15" customHeight="1">
+      <c r="A48" s="14" t="inlineStr">
         <is>
           <t>Jeux à la mi-temps</t>
         </is>
       </c>
-      <c r="C49" s="16" t="inlineStr"/>
-      <c r="D49" s="16" t="inlineStr"/>
-      <c r="E49" s="16" t="inlineStr"/>
-      <c r="F49" s="16" t="inlineStr"/>
-      <c r="G49" s="16" t="inlineStr"/>
-      <c r="H49" s="16" t="inlineStr"/>
-    </row>
-    <row r="50" ht="13" customHeight="1">
+      <c r="C48" s="15" t="inlineStr"/>
+      <c r="D48" s="15" t="inlineStr"/>
+      <c r="E48" s="15" t="inlineStr"/>
+      <c r="F48" s="15" t="inlineStr"/>
+      <c r="G48" s="15" t="inlineStr"/>
+      <c r="H48" s="15" t="inlineStr"/>
+    </row>
+    <row r="49" ht="10" customHeight="1">
+      <c r="A49" s="16" t="inlineStr">
+        <is>
+          <t>Animation proposée quand programmée (quiz, défis, jeux…)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="15" customHeight="1">
       <c r="A50" s="17" t="inlineStr">
         <is>
-          <t>Animation proposée quand programmée (quiz, défis, jeux…)</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="20" customHeight="1">
-      <c r="A51" s="18" t="inlineStr">
-        <is>
           <t>Relation clients</t>
         </is>
       </c>
-      <c r="C51" s="19" t="inlineStr"/>
-      <c r="D51" s="19" t="inlineStr"/>
-      <c r="E51" s="19" t="inlineStr"/>
-      <c r="F51" s="19" t="inlineStr"/>
-      <c r="G51" s="19" t="inlineStr"/>
-      <c r="H51" s="19" t="inlineStr"/>
-    </row>
-    <row r="52" ht="13" customHeight="1">
-      <c r="A52" s="20" t="inlineStr">
+      <c r="C50" s="18" t="inlineStr"/>
+      <c r="D50" s="18" t="inlineStr"/>
+      <c r="E50" s="18" t="inlineStr"/>
+      <c r="F50" s="18" t="inlineStr"/>
+      <c r="G50" s="18" t="inlineStr"/>
+      <c r="H50" s="18" t="inlineStr"/>
+    </row>
+    <row r="51" ht="10" customHeight="1">
+      <c r="A51" s="19" t="inlineStr">
         <is>
           <t>Discussions avec les joueurs/équipes, accueil, disponibilité</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="20" customHeight="1">
-      <c r="A53" s="15" t="inlineStr">
+    <row r="52" ht="15" customHeight="1">
+      <c r="A52" s="14" t="inlineStr">
         <is>
           <t>Ambiance de la soirée</t>
         </is>
       </c>
-      <c r="C53" s="16" t="inlineStr"/>
-      <c r="D53" s="16" t="inlineStr"/>
-      <c r="E53" s="16" t="inlineStr"/>
-      <c r="F53" s="16" t="inlineStr"/>
-      <c r="G53" s="16" t="inlineStr"/>
-      <c r="H53" s="16" t="inlineStr"/>
-    </row>
-    <row r="54" ht="13" customHeight="1">
-      <c r="A54" s="17" t="inlineStr">
+      <c r="C52" s="15" t="inlineStr"/>
+      <c r="D52" s="15" t="inlineStr"/>
+      <c r="E52" s="15" t="inlineStr"/>
+      <c r="F52" s="15" t="inlineStr"/>
+      <c r="G52" s="15" t="inlineStr"/>
+      <c r="H52" s="15" t="inlineStr"/>
+    </row>
+    <row r="53" ht="10" customHeight="1">
+      <c r="A53" s="16" t="inlineStr">
         <is>
           <t>Contribue à une bonne atmosphère, dynamise la soirée</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="18" customHeight="1">
-      <c r="A55" s="4" t="inlineStr">
+    <row r="54" ht="14" customHeight="1">
+      <c r="A54" s="4" t="inlineStr">
         <is>
           <t>SITUATIONS À REVOIR (VIDÉO)</t>
         </is>
       </c>
-      <c r="B55" s="5" t="n"/>
-      <c r="C55" s="5" t="n"/>
-      <c r="D55" s="5" t="n"/>
-      <c r="E55" s="5" t="n"/>
-      <c r="F55" s="5" t="n"/>
-      <c r="G55" s="5" t="n"/>
-      <c r="H55" s="5" t="n"/>
-    </row>
-    <row r="56" ht="14" customHeight="1">
-      <c r="A56" s="12" t="inlineStr">
+      <c r="B54" s="5" t="n"/>
+      <c r="C54" s="5" t="n"/>
+      <c r="D54" s="5" t="n"/>
+      <c r="E54" s="5" t="n"/>
+      <c r="F54" s="5" t="n"/>
+      <c r="G54" s="5" t="n"/>
+      <c r="H54" s="5" t="n"/>
+    </row>
+    <row r="55" ht="12" customHeight="1">
+      <c r="A55" s="11" t="inlineStr">
         <is>
           <t>Min.</t>
         </is>
       </c>
-      <c r="B56" s="6" t="inlineStr">
+      <c r="B55" s="20" t="inlineStr">
         <is>
           <t>Description de la situation</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="18" customHeight="1">
-      <c r="A57" s="16" t="inlineStr"/>
-      <c r="B57" s="7" t="inlineStr"/>
-    </row>
-    <row r="58" ht="18" customHeight="1">
-      <c r="A58" s="19" t="inlineStr"/>
+    <row r="56" ht="15" customHeight="1">
+      <c r="A56" s="15" t="inlineStr"/>
+      <c r="B56" s="21" t="inlineStr"/>
+    </row>
+    <row r="57" ht="15" customHeight="1">
+      <c r="A57" s="18" t="inlineStr"/>
+      <c r="B57" s="22" t="inlineStr"/>
+    </row>
+    <row r="58" ht="15" customHeight="1">
+      <c r="A58" s="15" t="inlineStr"/>
       <c r="B58" s="21" t="inlineStr"/>
     </row>
-    <row r="59" ht="18" customHeight="1">
-      <c r="A59" s="16" t="inlineStr"/>
-      <c r="B59" s="7" t="inlineStr"/>
-    </row>
-    <row r="60" ht="18" customHeight="1">
-      <c r="A60" s="19" t="inlineStr"/>
-      <c r="B60" s="21" t="inlineStr"/>
-    </row>
-    <row r="61" ht="18" customHeight="1">
-      <c r="A61" s="4" t="inlineStr">
+    <row r="59" ht="14" customHeight="1">
+      <c r="A59" s="4" t="inlineStr">
         <is>
           <t>BILAN</t>
         </is>
       </c>
-      <c r="B61" s="5" t="n"/>
-      <c r="C61" s="5" t="n"/>
-      <c r="D61" s="5" t="n"/>
-      <c r="E61" s="5" t="n"/>
-      <c r="F61" s="5" t="n"/>
-      <c r="G61" s="5" t="n"/>
-      <c r="H61" s="5" t="n"/>
-    </row>
-    <row r="62" ht="14" customHeight="1">
-      <c r="A62" s="22" t="inlineStr">
+      <c r="B59" s="5" t="n"/>
+      <c r="C59" s="5" t="n"/>
+      <c r="D59" s="5" t="n"/>
+      <c r="E59" s="5" t="n"/>
+      <c r="F59" s="5" t="n"/>
+      <c r="G59" s="5" t="n"/>
+      <c r="H59" s="5" t="n"/>
+    </row>
+    <row r="60" ht="12" customHeight="1">
+      <c r="A60" s="23" t="inlineStr">
         <is>
           <t>POINTS POSITIFS</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="18" customHeight="1">
-      <c r="A63" s="23" t="inlineStr"/>
-    </row>
-    <row r="64" ht="18" customHeight="1">
-      <c r="A64" s="24" t="inlineStr"/>
-    </row>
-    <row r="65" ht="14" customHeight="1">
-      <c r="A65" s="25" t="inlineStr">
+    <row r="61" ht="30" customHeight="1">
+      <c r="A61" s="24" t="inlineStr"/>
+    </row>
+    <row r="62" ht="12" customHeight="1">
+      <c r="A62" s="25" t="inlineStr">
         <is>
           <t>AXES D'AMÉLIORATION</t>
         </is>
       </c>
     </row>
-    <row r="66" ht="18" customHeight="1">
-      <c r="A66" s="23" t="inlineStr"/>
-    </row>
-    <row r="67" ht="18" customHeight="1">
-      <c r="A67" s="24" t="inlineStr"/>
-    </row>
-    <row r="68" ht="14" customHeight="1">
-      <c r="A68" s="11" t="inlineStr">
+    <row r="63" ht="30" customHeight="1">
+      <c r="A63" s="24" t="inlineStr"/>
+    </row>
+    <row r="64" ht="12" customHeight="1">
+      <c r="A64" s="10" t="inlineStr">
         <is>
           <t>COMMENTAIRE GÉNÉRAL</t>
         </is>
       </c>
     </row>
-    <row r="69" ht="18" customHeight="1">
-      <c r="A69" s="23" t="inlineStr"/>
-    </row>
-    <row r="70" ht="18" customHeight="1">
-      <c r="A70" s="24" t="inlineStr"/>
+    <row r="65" ht="30" customHeight="1">
+      <c r="A65" s="24" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="26" t="n"/>
+      <c r="B66" s="26" t="n"/>
+      <c r="C66" s="26" t="n"/>
+      <c r="D66" s="26" t="n"/>
+      <c r="E66" s="26" t="n"/>
+      <c r="F66" s="26" t="n"/>
+      <c r="G66" s="26" t="n"/>
+      <c r="H66" s="26" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="26" t="n"/>
+      <c r="B67" s="26" t="n"/>
+      <c r="C67" s="26" t="n"/>
+      <c r="D67" s="26" t="n"/>
+      <c r="E67" s="26" t="n"/>
+      <c r="F67" s="26" t="n"/>
+      <c r="G67" s="26" t="n"/>
+      <c r="H67" s="26" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="26" t="n"/>
+      <c r="B68" s="26" t="n"/>
+      <c r="C68" s="26" t="n"/>
+      <c r="D68" s="26" t="n"/>
+      <c r="E68" s="26" t="n"/>
+      <c r="F68" s="26" t="n"/>
+      <c r="G68" s="26" t="n"/>
+      <c r="H68" s="26" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="26" t="n"/>
+      <c r="B69" s="26" t="n"/>
+      <c r="C69" s="26" t="n"/>
+      <c r="D69" s="26" t="n"/>
+      <c r="E69" s="26" t="n"/>
+      <c r="F69" s="26" t="n"/>
+      <c r="G69" s="26" t="n"/>
+      <c r="H69" s="26" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="70">
-    <mergeCell ref="A9:H9"/>
-    <mergeCell ref="A67:H67"/>
-    <mergeCell ref="A48:H48"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="A30:H30"/>
-    <mergeCell ref="A39:H39"/>
+  <mergeCells count="66">
+    <mergeCell ref="A48:B48"/>
+    <mergeCell ref="A30:B30"/>
     <mergeCell ref="F5:H5"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A49:B49"/>
-    <mergeCell ref="A51:B51"/>
+    <mergeCell ref="A15:H15"/>
+    <mergeCell ref="A59:H59"/>
+    <mergeCell ref="A24:H24"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A51:H51"/>
     <mergeCell ref="A64:H64"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="B55:H55"/>
     <mergeCell ref="B6:H6"/>
-    <mergeCell ref="A36:H36"/>
-    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A60:H60"/>
+    <mergeCell ref="A49:H49"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A45:H45"/>
     <mergeCell ref="A61:H61"/>
-    <mergeCell ref="A70:H70"/>
-    <mergeCell ref="A69:H69"/>
-    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A25:B25"/>
     <mergeCell ref="A65:H65"/>
-    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A41:B41"/>
     <mergeCell ref="A54:H54"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="A46:B46"/>
-    <mergeCell ref="A41:H41"/>
-    <mergeCell ref="A66:H66"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="A27:H27"/>
-    <mergeCell ref="B59:H59"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A18:H18"/>
-    <mergeCell ref="A50:H50"/>
-    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A37:H37"/>
+    <mergeCell ref="A46:H46"/>
+    <mergeCell ref="A50:B50"/>
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="A21:B21"/>
     <mergeCell ref="B5:D5"/>
-    <mergeCell ref="A21:H21"/>
-    <mergeCell ref="A55:H55"/>
+    <mergeCell ref="A26:H26"/>
     <mergeCell ref="B56:H56"/>
     <mergeCell ref="B58:H58"/>
-    <mergeCell ref="A33:B33"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A42:B42"/>
-    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="A42:H42"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A33:H33"/>
     <mergeCell ref="A47:H47"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="A23:B23"/>
     <mergeCell ref="B7:D7"/>
-    <mergeCell ref="A32:H32"/>
-    <mergeCell ref="B60:H60"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A53:B53"/>
-    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A22:H22"/>
+    <mergeCell ref="A17:H17"/>
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="A62:H62"/>
+    <mergeCell ref="A53:H53"/>
+    <mergeCell ref="A52:B52"/>
     <mergeCell ref="A29:H29"/>
+    <mergeCell ref="A35:H35"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A38:H38"/>
     <mergeCell ref="B57:H57"/>
-    <mergeCell ref="A20:H20"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A38:H38"/>
-    <mergeCell ref="A43:H43"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="A52:H52"/>
     <mergeCell ref="A63:H63"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A28:H28"/>
     <mergeCell ref="A13:H13"/>
-    <mergeCell ref="A44:B44"/>
-    <mergeCell ref="A68:H68"/>
+    <mergeCell ref="A19:H19"/>
+    <mergeCell ref="A44:H44"/>
     <mergeCell ref="F7:H7"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="A34:H34"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A31:H31"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A40:H40"/>
   </mergeCells>
-  <pageMargins left="0.3" right="0.3" top="0.3" bottom="0.3" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" fitToHeight="1" fitToWidth="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0" footer="0"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Arbitre : fusionner ambiance+clients, enlever concentration et ponctualité
- Fusionner Relation clients + Ambiance de la soirée en un seul critère
- Supprimer Concentration (Attitude)
- Retirer ponctualité de la description Présentation
- Appliqué sur HTML et Excel

https://claude.ai/code/session_01ELsd82FqhFHd9QHcP9yAqq
</commit_message>
<xml_diff>
--- a/Evaluation Arbitre - UrbanSoccer.xlsx
+++ b/Evaluation Arbitre - UrbanSoccer.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Évaluation Arbitre" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Évaluation Arbitre'!$A$1:$H$65</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Évaluation Arbitre'!$A$1:$H$61</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1177,7 +1177,7 @@
     <row r="40" ht="10" customHeight="1">
       <c r="A40" s="16" t="inlineStr">
         <is>
-          <t>Tenue correcte, ponctualité, équipement d'arbitre</t>
+          <t>Tenue correcte, équipement d'arbitre</t>
         </is>
       </c>
     </row>
@@ -1204,7 +1204,7 @@
     <row r="43" ht="15" customHeight="1">
       <c r="A43" s="14" t="inlineStr">
         <is>
-          <t>Concentration</t>
+          <t>Timing &amp; Gestion du temps</t>
         </is>
       </c>
       <c r="C43" s="15" t="inlineStr"/>
@@ -1217,48 +1217,48 @@
     <row r="44" ht="10" customHeight="1">
       <c r="A44" s="16" t="inlineStr">
         <is>
-          <t>Reste attentif du début à la fin, même sur les temps morts</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="15" customHeight="1">
-      <c r="A45" s="17" t="inlineStr">
-        <is>
-          <t>Timing &amp; Gestion du temps</t>
-        </is>
-      </c>
-      <c r="C45" s="18" t="inlineStr"/>
-      <c r="D45" s="18" t="inlineStr"/>
-      <c r="E45" s="18" t="inlineStr"/>
-      <c r="F45" s="18" t="inlineStr"/>
-      <c r="G45" s="18" t="inlineStr"/>
-      <c r="H45" s="18" t="inlineStr"/>
-    </row>
-    <row r="46" ht="10" customHeight="1">
-      <c r="A46" s="19" t="inlineStr">
-        <is>
           <t>Début des matchs à l'heure, durées de mi-temps, enchaînement</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="13" customHeight="1">
-      <c r="A47" s="12" t="inlineStr">
+    <row r="45" ht="13" customHeight="1">
+      <c r="A45" s="12" t="inlineStr">
         <is>
           <t>ANIMATION</t>
         </is>
       </c>
-      <c r="B47" s="13" t="n"/>
-      <c r="C47" s="13" t="n"/>
-      <c r="D47" s="13" t="n"/>
-      <c r="E47" s="13" t="n"/>
-      <c r="F47" s="13" t="n"/>
-      <c r="G47" s="13" t="n"/>
-      <c r="H47" s="13" t="n"/>
+      <c r="B45" s="13" t="n"/>
+      <c r="C45" s="13" t="n"/>
+      <c r="D45" s="13" t="n"/>
+      <c r="E45" s="13" t="n"/>
+      <c r="F45" s="13" t="n"/>
+      <c r="G45" s="13" t="n"/>
+      <c r="H45" s="13" t="n"/>
+    </row>
+    <row r="46" ht="15" customHeight="1">
+      <c r="A46" s="17" t="inlineStr">
+        <is>
+          <t>Jeux à la mi-temps</t>
+        </is>
+      </c>
+      <c r="C46" s="18" t="inlineStr"/>
+      <c r="D46" s="18" t="inlineStr"/>
+      <c r="E46" s="18" t="inlineStr"/>
+      <c r="F46" s="18" t="inlineStr"/>
+      <c r="G46" s="18" t="inlineStr"/>
+      <c r="H46" s="18" t="inlineStr"/>
+    </row>
+    <row r="47" ht="10" customHeight="1">
+      <c r="A47" s="19" t="inlineStr">
+        <is>
+          <t>Animation proposée quand programmée (quiz, défis, jeux…)</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="A48" s="14" t="inlineStr">
         <is>
-          <t>Jeux à la mi-temps</t>
+          <t>Relation clients &amp; Ambiance</t>
         </is>
       </c>
       <c r="C48" s="15" t="inlineStr"/>
@@ -1271,131 +1271,131 @@
     <row r="49" ht="10" customHeight="1">
       <c r="A49" s="16" t="inlineStr">
         <is>
-          <t>Animation proposée quand programmée (quiz, défis, jeux…)</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="15" customHeight="1">
-      <c r="A50" s="17" t="inlineStr">
-        <is>
-          <t>Relation clients</t>
-        </is>
-      </c>
-      <c r="C50" s="18" t="inlineStr"/>
-      <c r="D50" s="18" t="inlineStr"/>
-      <c r="E50" s="18" t="inlineStr"/>
-      <c r="F50" s="18" t="inlineStr"/>
-      <c r="G50" s="18" t="inlineStr"/>
-      <c r="H50" s="18" t="inlineStr"/>
-    </row>
-    <row r="51" ht="10" customHeight="1">
-      <c r="A51" s="19" t="inlineStr">
-        <is>
-          <t>Discussions avec les joueurs/équipes, accueil, disponibilité</t>
+          <t>Discussions joueurs/équipes, accueil, disponibilité, bonne atmosphère</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="14" customHeight="1">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>SITUATIONS À REVOIR (VIDÉO)</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n"/>
+      <c r="C50" s="5" t="n"/>
+      <c r="D50" s="5" t="n"/>
+      <c r="E50" s="5" t="n"/>
+      <c r="F50" s="5" t="n"/>
+      <c r="G50" s="5" t="n"/>
+      <c r="H50" s="5" t="n"/>
+    </row>
+    <row r="51" ht="12" customHeight="1">
+      <c r="A51" s="11" t="inlineStr">
+        <is>
+          <t>Min.</t>
+        </is>
+      </c>
+      <c r="B51" s="20" t="inlineStr">
+        <is>
+          <t>Description de la situation</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
-      <c r="A52" s="14" t="inlineStr">
-        <is>
-          <t>Ambiance de la soirée</t>
-        </is>
-      </c>
-      <c r="C52" s="15" t="inlineStr"/>
-      <c r="D52" s="15" t="inlineStr"/>
-      <c r="E52" s="15" t="inlineStr"/>
-      <c r="F52" s="15" t="inlineStr"/>
-      <c r="G52" s="15" t="inlineStr"/>
-      <c r="H52" s="15" t="inlineStr"/>
-    </row>
-    <row r="53" ht="10" customHeight="1">
-      <c r="A53" s="16" t="inlineStr">
-        <is>
-          <t>Contribue à une bonne atmosphère, dynamise la soirée</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="14" customHeight="1">
-      <c r="A54" s="4" t="inlineStr">
-        <is>
-          <t>SITUATIONS À REVOIR (VIDÉO)</t>
-        </is>
-      </c>
-      <c r="B54" s="5" t="n"/>
-      <c r="C54" s="5" t="n"/>
-      <c r="D54" s="5" t="n"/>
-      <c r="E54" s="5" t="n"/>
-      <c r="F54" s="5" t="n"/>
-      <c r="G54" s="5" t="n"/>
-      <c r="H54" s="5" t="n"/>
-    </row>
-    <row r="55" ht="12" customHeight="1">
-      <c r="A55" s="11" t="inlineStr">
-        <is>
-          <t>Min.</t>
-        </is>
-      </c>
-      <c r="B55" s="20" t="inlineStr">
-        <is>
-          <t>Description de la situation</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="15" customHeight="1">
-      <c r="A56" s="15" t="inlineStr"/>
-      <c r="B56" s="21" t="inlineStr"/>
-    </row>
-    <row r="57" ht="15" customHeight="1">
-      <c r="A57" s="18" t="inlineStr"/>
-      <c r="B57" s="22" t="inlineStr"/>
-    </row>
-    <row r="58" ht="15" customHeight="1">
-      <c r="A58" s="15" t="inlineStr"/>
-      <c r="B58" s="21" t="inlineStr"/>
-    </row>
-    <row r="59" ht="14" customHeight="1">
-      <c r="A59" s="4" t="inlineStr">
+      <c r="A52" s="15" t="inlineStr"/>
+      <c r="B52" s="21" t="inlineStr"/>
+    </row>
+    <row r="53" ht="15" customHeight="1">
+      <c r="A53" s="18" t="inlineStr"/>
+      <c r="B53" s="22" t="inlineStr"/>
+    </row>
+    <row r="54" ht="15" customHeight="1">
+      <c r="A54" s="15" t="inlineStr"/>
+      <c r="B54" s="21" t="inlineStr"/>
+    </row>
+    <row r="55" ht="14" customHeight="1">
+      <c r="A55" s="4" t="inlineStr">
         <is>
           <t>BILAN</t>
         </is>
       </c>
-      <c r="B59" s="5" t="n"/>
-      <c r="C59" s="5" t="n"/>
-      <c r="D59" s="5" t="n"/>
-      <c r="E59" s="5" t="n"/>
-      <c r="F59" s="5" t="n"/>
-      <c r="G59" s="5" t="n"/>
-      <c r="H59" s="5" t="n"/>
+      <c r="B55" s="5" t="n"/>
+      <c r="C55" s="5" t="n"/>
+      <c r="D55" s="5" t="n"/>
+      <c r="E55" s="5" t="n"/>
+      <c r="F55" s="5" t="n"/>
+      <c r="G55" s="5" t="n"/>
+      <c r="H55" s="5" t="n"/>
+    </row>
+    <row r="56" ht="12" customHeight="1">
+      <c r="A56" s="23" t="inlineStr">
+        <is>
+          <t>POINTS POSITIFS</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="30" customHeight="1">
+      <c r="A57" s="24" t="inlineStr"/>
+    </row>
+    <row r="58" ht="12" customHeight="1">
+      <c r="A58" s="25" t="inlineStr">
+        <is>
+          <t>AXES D'AMÉLIORATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="30" customHeight="1">
+      <c r="A59" s="24" t="inlineStr"/>
     </row>
     <row r="60" ht="12" customHeight="1">
-      <c r="A60" s="23" t="inlineStr">
-        <is>
-          <t>POINTS POSITIFS</t>
+      <c r="A60" s="10" t="inlineStr">
+        <is>
+          <t>COMMENTAIRE GÉNÉRAL</t>
         </is>
       </c>
     </row>
     <row r="61" ht="30" customHeight="1">
       <c r="A61" s="24" t="inlineStr"/>
     </row>
-    <row r="62" ht="12" customHeight="1">
-      <c r="A62" s="25" t="inlineStr">
-        <is>
-          <t>AXES D'AMÉLIORATION</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="30" customHeight="1">
-      <c r="A63" s="24" t="inlineStr"/>
-    </row>
-    <row r="64" ht="12" customHeight="1">
-      <c r="A64" s="10" t="inlineStr">
-        <is>
-          <t>COMMENTAIRE GÉNÉRAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="30" customHeight="1">
-      <c r="A65" s="24" t="inlineStr"/>
+    <row r="62">
+      <c r="A62" s="26" t="n"/>
+      <c r="B62" s="26" t="n"/>
+      <c r="C62" s="26" t="n"/>
+      <c r="D62" s="26" t="n"/>
+      <c r="E62" s="26" t="n"/>
+      <c r="F62" s="26" t="n"/>
+      <c r="G62" s="26" t="n"/>
+      <c r="H62" s="26" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="26" t="n"/>
+      <c r="B63" s="26" t="n"/>
+      <c r="C63" s="26" t="n"/>
+      <c r="D63" s="26" t="n"/>
+      <c r="E63" s="26" t="n"/>
+      <c r="F63" s="26" t="n"/>
+      <c r="G63" s="26" t="n"/>
+      <c r="H63" s="26" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="26" t="n"/>
+      <c r="B64" s="26" t="n"/>
+      <c r="C64" s="26" t="n"/>
+      <c r="D64" s="26" t="n"/>
+      <c r="E64" s="26" t="n"/>
+      <c r="F64" s="26" t="n"/>
+      <c r="G64" s="26" t="n"/>
+      <c r="H64" s="26" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="26" t="n"/>
+      <c r="B65" s="26" t="n"/>
+      <c r="C65" s="26" t="n"/>
+      <c r="D65" s="26" t="n"/>
+      <c r="E65" s="26" t="n"/>
+      <c r="F65" s="26" t="n"/>
+      <c r="G65" s="26" t="n"/>
+      <c r="H65" s="26" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="26" t="n"/>
@@ -1438,7 +1438,7 @@
       <c r="H69" s="26" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="66">
+  <mergeCells count="62">
     <mergeCell ref="A48:B48"/>
     <mergeCell ref="A30:B30"/>
     <mergeCell ref="F5:H5"/>
@@ -1446,32 +1446,31 @@
     <mergeCell ref="A59:H59"/>
     <mergeCell ref="A24:H24"/>
     <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A51:H51"/>
-    <mergeCell ref="A64:H64"/>
-    <mergeCell ref="A45:B45"/>
-    <mergeCell ref="B55:H55"/>
     <mergeCell ref="B6:H6"/>
     <mergeCell ref="A36:B36"/>
     <mergeCell ref="A60:H60"/>
     <mergeCell ref="A49:H49"/>
     <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A45:H45"/>
+    <mergeCell ref="B51:H51"/>
     <mergeCell ref="A61:H61"/>
     <mergeCell ref="A16:B16"/>
     <mergeCell ref="A25:B25"/>
-    <mergeCell ref="A65:H65"/>
     <mergeCell ref="A41:B41"/>
-    <mergeCell ref="A54:H54"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="B54:H54"/>
     <mergeCell ref="A18:B18"/>
     <mergeCell ref="A27:B27"/>
     <mergeCell ref="A37:H37"/>
-    <mergeCell ref="A46:H46"/>
-    <mergeCell ref="A50:B50"/>
     <mergeCell ref="A12:H12"/>
+    <mergeCell ref="A50:H50"/>
+    <mergeCell ref="A56:H56"/>
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="A26:H26"/>
-    <mergeCell ref="B56:H56"/>
-    <mergeCell ref="B58:H58"/>
+    <mergeCell ref="A55:H55"/>
+    <mergeCell ref="B52:H52"/>
+    <mergeCell ref="A57:H57"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A42:H42"/>
     <mergeCell ref="A32:B32"/>
@@ -1484,21 +1483,18 @@
     <mergeCell ref="A22:H22"/>
     <mergeCell ref="A17:H17"/>
     <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A62:H62"/>
-    <mergeCell ref="A53:H53"/>
-    <mergeCell ref="A52:B52"/>
     <mergeCell ref="A29:H29"/>
     <mergeCell ref="A35:H35"/>
     <mergeCell ref="A43:B43"/>
     <mergeCell ref="A20:H20"/>
     <mergeCell ref="A38:H38"/>
-    <mergeCell ref="B57:H57"/>
-    <mergeCell ref="A63:H63"/>
+    <mergeCell ref="B53:H53"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A28:H28"/>
     <mergeCell ref="A13:H13"/>
     <mergeCell ref="A19:H19"/>
     <mergeCell ref="A44:H44"/>
+    <mergeCell ref="A58:H58"/>
     <mergeCell ref="F7:H7"/>
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="A31:H31"/>

</xml_diff>